<commit_message>
Fill October electricity bill amounts for 6/11/13F
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FM2YJqCagBbEuBH1oLpGAS
</commit_message>
<xml_diff>
--- a/out/전기세_지출결의서_26.10.xlsx
+++ b/out/전기세_지출결의서_26.10.xlsx
@@ -782,29 +782,14 @@
     <author>경영기획실</author>
   </authors>
   <commentList>
-    <comment ref="D2" authorId="0" shapeId="0">
-      <text>
-        <t>10월 고지서 공급가 입력</t>
-      </text>
-    </comment>
     <comment ref="D5" authorId="0" shapeId="0">
       <text>
         <t>단수차이 자동 조정(총액-다른 부서 합)</t>
       </text>
     </comment>
-    <comment ref="D8" authorId="0" shapeId="0">
-      <text>
-        <t>10월 고지서 공급가 입력</t>
-      </text>
-    </comment>
     <comment ref="D14" authorId="0" shapeId="0">
       <text>
         <t>단수차이 자동 조정(총액-다른 부서 합)</t>
-      </text>
-    </comment>
-    <comment ref="D17" authorId="0" shapeId="0">
-      <text>
-        <t>10월 고지서 공급가 입력</t>
       </text>
     </comment>
     <comment ref="D23" authorId="0" shapeId="0">
@@ -2890,8 +2875,13 @@
       </c>
       <c r="B2" s="55" t="n"/>
       <c r="C2" s="56" t="n"/>
-      <c r="D2" s="65" t="n"/>
-      <c r="E2" s="65" t="n"/>
+      <c r="D2" s="79">
+        <f>294223+7940-5</f>
+        <v/>
+      </c>
+      <c r="E2" s="79" t="n">
+        <v>29422</v>
+      </c>
       <c r="F2" s="66">
         <f>D2+E2</f>
         <v/>
@@ -3149,8 +3139,13 @@
       </c>
       <c r="B8" s="55" t="n"/>
       <c r="C8" s="56" t="n"/>
-      <c r="D8" s="65" t="n"/>
-      <c r="E8" s="65" t="n"/>
+      <c r="D8" s="79">
+        <f>276764+7470</f>
+        <v/>
+      </c>
+      <c r="E8" s="79" t="n">
+        <v>27676</v>
+      </c>
       <c r="F8" s="66">
         <f>D8+E8</f>
         <v/>
@@ -3572,8 +3567,13 @@
       </c>
       <c r="B17" s="55" t="n"/>
       <c r="C17" s="56" t="n"/>
-      <c r="D17" s="65" t="n"/>
-      <c r="E17" s="65" t="n"/>
+      <c r="D17" s="79">
+        <f>308764+8330</f>
+        <v/>
+      </c>
+      <c r="E17" s="79" t="n">
+        <v>30876</v>
+      </c>
       <c r="F17" s="66">
         <f>D17+E17</f>
         <v/>
@@ -8913,10 +8913,10 @@
     <col width="12.875" customWidth="1" style="53" min="4" max="4"/>
     <col width="16.75" customWidth="1" style="63" min="5" max="5"/>
     <col width="15.25" customWidth="1" style="53" min="6" max="7"/>
-    <col hidden="1" style="53" min="9" max="10"/>
+    <col hidden="1" width="13" customWidth="1" style="53" min="9" max="10"/>
     <col hidden="1" width="11.375" customWidth="1" style="53" min="11" max="11"/>
     <col hidden="1" width="18.625" customWidth="1" style="53" min="12" max="12"/>
-    <col hidden="1" style="53" min="13" max="14"/>
+    <col hidden="1" width="13" customWidth="1" style="53" min="13" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="53" thickBot="1">
@@ -15201,10 +15201,10 @@
     <col width="12.875" customWidth="1" style="53" min="4" max="4"/>
     <col width="16.75" customWidth="1" style="63" min="5" max="5"/>
     <col width="15.25" customWidth="1" style="53" min="6" max="7"/>
-    <col hidden="1" style="53" min="9" max="10"/>
+    <col hidden="1" width="13" customWidth="1" style="53" min="9" max="10"/>
     <col hidden="1" width="11.375" customWidth="1" style="53" min="11" max="11"/>
     <col hidden="1" width="12.75" customWidth="1" style="53" min="12" max="12"/>
-    <col hidden="1" style="53" min="13" max="14"/>
+    <col hidden="1" width="13" customWidth="1" style="53" min="13" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="53" thickBot="1">

</xml_diff>

<commit_message>
Add 이종원 (경영기획실, 13F) to October electricity roster
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FM2YJqCagBbEuBH1oLpGAS
</commit_message>
<xml_diff>
--- a/out/전기세_지출결의서_26.10.xlsx
+++ b/out/전기세_지출결의서_26.10.xlsx
@@ -1418,24 +1418,20 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C12" s="22" t="inlineStr">
-        <is>
-          <t>R&amp;D본부</t>
-        </is>
-      </c>
+      <c r="C12" s="22" t="n"/>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>표준모델 개발TF</t>
+          <t>경영기획실</t>
         </is>
       </c>
       <c r="E12" s="22" t="inlineStr">
         <is>
-          <t>최진달미</t>
+          <t>이종원</t>
         </is>
       </c>
       <c r="F12" s="22" t="inlineStr">
         <is>
-          <t>수석연구위원</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
@@ -1460,12 +1456,12 @@
       </c>
       <c r="E13" s="22" t="inlineStr">
         <is>
-          <t>오한솔</t>
+          <t>최진달미</t>
         </is>
       </c>
       <c r="F13" s="22" t="inlineStr">
         <is>
-          <t>연구원</t>
+          <t>수석연구위원</t>
         </is>
       </c>
     </row>
@@ -1485,49 +1481,53 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>D-LAB 2실</t>
+          <t>표준모델 개발TF</t>
         </is>
       </c>
       <c r="E14" s="22" t="inlineStr">
         <is>
-          <t>최수지</t>
+          <t>오한솔</t>
         </is>
       </c>
       <c r="F14" s="22" t="inlineStr">
         <is>
-          <t>책임연구원</t>
+          <t>연구원</t>
         </is>
       </c>
     </row>
     <row r="15" ht="13.5" customFormat="1" customHeight="1" s="11">
       <c r="A15" s="22" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>6층</t>
-        </is>
-      </c>
-      <c r="C15" s="22" t="n"/>
+          <t>13층</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>R&amp;D본부</t>
+        </is>
+      </c>
       <c r="D15" s="22" t="inlineStr">
         <is>
-          <t>신사업개발실</t>
+          <t>D-LAB 2실</t>
         </is>
       </c>
       <c r="E15" s="22" t="inlineStr">
         <is>
-          <t>김태우</t>
+          <t>최수지</t>
         </is>
       </c>
       <c r="F15" s="22" t="inlineStr">
         <is>
-          <t>상무</t>
+          <t>책임연구원</t>
         </is>
       </c>
     </row>
     <row r="16" ht="13.5" customHeight="1" s="53">
       <c r="A16" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
@@ -1542,18 +1542,18 @@
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>김순성</t>
+          <t>김태우</t>
         </is>
       </c>
       <c r="F16" s="22" t="inlineStr">
         <is>
-          <t>고문</t>
+          <t>상무</t>
         </is>
       </c>
     </row>
     <row r="17" ht="13.5" customHeight="1" s="53">
       <c r="A17" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B17" s="22" t="inlineStr">
         <is>
@@ -1568,18 +1568,18 @@
       </c>
       <c r="E17" s="22" t="inlineStr">
         <is>
-          <t>박종철</t>
+          <t>김순성</t>
         </is>
       </c>
       <c r="F17" s="22" t="inlineStr">
         <is>
-          <t>이사보</t>
+          <t>고문</t>
         </is>
       </c>
     </row>
     <row r="18" ht="13.5" customHeight="1" s="53">
       <c r="A18" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
@@ -1594,48 +1594,44 @@
       </c>
       <c r="E18" s="22" t="inlineStr">
         <is>
-          <t>이정진</t>
+          <t>박종철</t>
         </is>
       </c>
       <c r="F18" s="22" t="inlineStr">
         <is>
-          <t>부장</t>
+          <t>이사보</t>
         </is>
       </c>
     </row>
     <row r="19" ht="13.5" customFormat="1" customHeight="1" s="11">
       <c r="A19" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>11층</t>
-        </is>
-      </c>
-      <c r="C19" s="22" t="inlineStr">
-        <is>
-          <t>사업관리본부</t>
-        </is>
-      </c>
+          <t>6층</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="n"/>
       <c r="D19" s="22" t="inlineStr">
         <is>
-          <t>설계실</t>
+          <t>신사업개발실</t>
         </is>
       </c>
       <c r="E19" s="22" t="inlineStr">
         <is>
-          <t>오진택</t>
+          <t>이정진</t>
         </is>
       </c>
       <c r="F19" s="22" t="inlineStr">
         <is>
-          <t>부사장</t>
+          <t>부장</t>
         </is>
       </c>
     </row>
     <row r="20" ht="13.5" customHeight="1" s="53">
       <c r="A20" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
@@ -1654,18 +1650,18 @@
       </c>
       <c r="E20" s="22" t="inlineStr">
         <is>
-          <t>최우제</t>
+          <t>오진택</t>
         </is>
       </c>
       <c r="F20" s="22" t="inlineStr">
         <is>
-          <t>상무</t>
+          <t>부사장</t>
         </is>
       </c>
     </row>
     <row r="21" ht="13.5" customFormat="1" customHeight="1" s="11">
       <c r="A21" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
@@ -1684,18 +1680,18 @@
       </c>
       <c r="E21" s="22" t="inlineStr">
         <is>
-          <t>김채영</t>
+          <t>최우제</t>
         </is>
       </c>
       <c r="F21" s="22" t="inlineStr">
         <is>
-          <t>이사보</t>
+          <t>상무</t>
         </is>
       </c>
     </row>
     <row r="22" ht="13.5" customFormat="1" customHeight="1" s="11">
       <c r="A22" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
@@ -1714,18 +1710,18 @@
       </c>
       <c r="E22" s="22" t="inlineStr">
         <is>
-          <t>김태은</t>
+          <t>김채영</t>
         </is>
       </c>
       <c r="F22" s="22" t="inlineStr">
         <is>
-          <t>과장</t>
+          <t>이사보</t>
         </is>
       </c>
     </row>
     <row r="23" ht="13.5" customFormat="1" customHeight="1" s="11">
       <c r="A23" s="22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23" s="22" t="inlineStr">
         <is>
@@ -1744,18 +1740,18 @@
       </c>
       <c r="E23" s="22" t="inlineStr">
         <is>
-          <t>김민호</t>
+          <t>김태은</t>
         </is>
       </c>
       <c r="F23" s="22" t="inlineStr">
         <is>
-          <t>대리</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
     <row r="24" ht="13.5" customHeight="1" s="53">
       <c r="A24" s="22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
@@ -1774,18 +1770,18 @@
       </c>
       <c r="E24" s="22" t="inlineStr">
         <is>
-          <t>이수영</t>
+          <t>김민호</t>
         </is>
       </c>
       <c r="F24" s="22" t="inlineStr">
         <is>
-          <t>주임</t>
+          <t>대리</t>
         </is>
       </c>
     </row>
     <row r="25" ht="14.25" customFormat="1" customHeight="1" s="11" thickBot="1">
       <c r="A25" s="22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
@@ -1804,18 +1800,18 @@
       </c>
       <c r="E25" s="22" t="inlineStr">
         <is>
-          <t>최수용</t>
+          <t>이수영</t>
         </is>
       </c>
       <c r="F25" s="22" t="inlineStr">
         <is>
-          <t>사원</t>
+          <t>주임</t>
         </is>
       </c>
     </row>
     <row r="26" ht="14.25" customFormat="1" customHeight="1" s="11" thickTop="1">
       <c r="A26" s="22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
@@ -1829,23 +1825,23 @@
       </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>설계실</t>
         </is>
       </c>
       <c r="E26" s="22" t="inlineStr">
         <is>
-          <t>김동우</t>
+          <t>최수용</t>
         </is>
       </c>
       <c r="F26" s="22" t="inlineStr">
         <is>
-          <t>부사장</t>
+          <t>사원</t>
         </is>
       </c>
     </row>
     <row r="27" ht="13.5" customFormat="1" customHeight="1" s="11">
       <c r="A27" s="22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
@@ -1864,18 +1860,18 @@
       </c>
       <c r="E27" s="22" t="inlineStr">
         <is>
-          <t>이성규</t>
+          <t>김동우</t>
         </is>
       </c>
       <c r="F27" s="22" t="inlineStr">
         <is>
-          <t>차장</t>
+          <t>부사장</t>
         </is>
       </c>
     </row>
     <row r="28" ht="13.5" customHeight="1" s="53">
       <c r="A28" s="22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
@@ -1894,7 +1890,7 @@
       </c>
       <c r="E28" s="22" t="inlineStr">
         <is>
-          <t>이강호</t>
+          <t>이성규</t>
         </is>
       </c>
       <c r="F28" s="22" t="inlineStr">
@@ -1905,7 +1901,7 @@
     </row>
     <row r="29" ht="13.5" customHeight="1" s="53">
       <c r="A29" s="22" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
@@ -1924,18 +1920,18 @@
       </c>
       <c r="E29" s="22" t="inlineStr">
         <is>
-          <t>김동규</t>
+          <t>이강호</t>
         </is>
       </c>
       <c r="F29" s="22" t="inlineStr">
         <is>
-          <t>부장</t>
+          <t>차장</t>
         </is>
       </c>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="53">
       <c r="A30" s="22" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
@@ -1949,23 +1945,23 @@
       </c>
       <c r="D30" s="22" t="inlineStr">
         <is>
-          <t>사업관리1실</t>
+          <t>사업관리본부</t>
         </is>
       </c>
       <c r="E30" s="22" t="inlineStr">
         <is>
-          <t>김승현</t>
+          <t>김동규</t>
         </is>
       </c>
       <c r="F30" s="22" t="inlineStr">
         <is>
-          <t>상무</t>
+          <t>부장</t>
         </is>
       </c>
     </row>
     <row r="31" ht="13.5" customHeight="1" s="53">
       <c r="A31" s="22" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
@@ -1984,18 +1980,18 @@
       </c>
       <c r="E31" s="22" t="inlineStr">
         <is>
-          <t>조지은</t>
+          <t>김승현</t>
         </is>
       </c>
       <c r="F31" s="22" t="inlineStr">
         <is>
-          <t>이사보</t>
+          <t>상무</t>
         </is>
       </c>
     </row>
     <row r="32" ht="13.5" customHeight="1" s="53">
       <c r="A32" s="22" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
@@ -2014,18 +2010,18 @@
       </c>
       <c r="E32" s="22" t="inlineStr">
         <is>
-          <t>이예솔</t>
+          <t>조지은</t>
         </is>
       </c>
       <c r="F32" s="22" t="inlineStr">
         <is>
-          <t>과장</t>
+          <t>이사보</t>
         </is>
       </c>
     </row>
     <row r="33" ht="13.5" customHeight="1" s="53">
       <c r="A33" s="22" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
@@ -2044,7 +2040,7 @@
       </c>
       <c r="E33" s="22" t="inlineStr">
         <is>
-          <t>류승호</t>
+          <t>이예솔</t>
         </is>
       </c>
       <c r="F33" s="22" t="inlineStr">
@@ -2055,7 +2051,7 @@
     </row>
     <row r="34" ht="13.5" customHeight="1" s="53">
       <c r="A34" s="22" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
@@ -2069,23 +2065,23 @@
       </c>
       <c r="D34" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>사업관리1실</t>
         </is>
       </c>
       <c r="E34" s="22" t="inlineStr">
         <is>
-          <t>주현철</t>
+          <t>류승호</t>
         </is>
       </c>
       <c r="F34" s="22" t="inlineStr">
         <is>
-          <t>상무</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
     <row r="35" ht="13.5" customHeight="1" s="53">
       <c r="A35" s="22" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
@@ -2104,18 +2100,18 @@
       </c>
       <c r="E35" s="22" t="inlineStr">
         <is>
-          <t>이완구</t>
+          <t>주현철</t>
         </is>
       </c>
       <c r="F35" s="22" t="inlineStr">
         <is>
-          <t>이사보</t>
+          <t>상무</t>
         </is>
       </c>
     </row>
     <row r="36" ht="13.5" customHeight="1" s="53">
       <c r="A36" s="22" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B36" s="22" t="inlineStr">
         <is>
@@ -2134,18 +2130,18 @@
       </c>
       <c r="E36" s="22" t="inlineStr">
         <is>
-          <t>황진욱</t>
+          <t>이완구</t>
         </is>
       </c>
       <c r="F36" s="22" t="inlineStr">
         <is>
-          <t>대리</t>
+          <t>이사보</t>
         </is>
       </c>
     </row>
     <row r="37" ht="13.5" customHeight="1" s="53">
       <c r="A37" s="22" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B37" s="22" t="inlineStr">
         <is>
@@ -2164,18 +2160,18 @@
       </c>
       <c r="E37" s="22" t="inlineStr">
         <is>
-          <t>문광정</t>
+          <t>황진욱</t>
         </is>
       </c>
       <c r="F37" s="22" t="inlineStr">
         <is>
-          <t>부장</t>
+          <t>대리</t>
         </is>
       </c>
     </row>
     <row r="38" ht="13.5" customFormat="1" customHeight="1" s="11">
       <c r="A38" s="22" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B38" s="22" t="inlineStr">
         <is>
@@ -2194,19 +2190,19 @@
       </c>
       <c r="E38" s="22" t="inlineStr">
         <is>
-          <t>정연석</t>
+          <t>문광정</t>
         </is>
       </c>
       <c r="F38" s="22" t="inlineStr">
         <is>
-          <t>대리</t>
+          <t>부장</t>
         </is>
       </c>
       <c r="G38" s="10" t="n"/>
     </row>
     <row r="39" ht="13.5" customFormat="1" customHeight="1" s="11">
       <c r="A39" s="22" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B39" s="22" t="inlineStr">
         <is>
@@ -2225,7 +2221,7 @@
       </c>
       <c r="E39" s="22" t="inlineStr">
         <is>
-          <t>김진규</t>
+          <t>정연석</t>
         </is>
       </c>
       <c r="F39" s="22" t="inlineStr">
@@ -2237,35 +2233,64 @@
     </row>
     <row r="40" ht="14.25" customHeight="1" s="53" thickBot="1">
       <c r="A40" s="22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>11층</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>사업관리본부</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>사업관리2실</t>
+        </is>
+      </c>
+      <c r="E40" s="22" t="inlineStr">
+        <is>
+          <t>김진규</t>
+        </is>
+      </c>
+      <c r="F40" s="22" t="inlineStr">
+        <is>
+          <t>대리</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="17.25" customHeight="1" s="53" thickTop="1">
+      <c r="A41" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B41" s="22" t="inlineStr">
         <is>
           <t>11층</t>
         </is>
       </c>
-      <c r="C40" s="22" t="inlineStr">
+      <c r="C41" s="22" t="inlineStr">
         <is>
           <t>사업관리본부</t>
         </is>
       </c>
-      <c r="D40" s="22" t="inlineStr">
+      <c r="D41" s="22" t="inlineStr">
         <is>
           <t>사업관리2실</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr">
+      <c r="E41" s="22" t="inlineStr">
         <is>
           <t>연지현</t>
         </is>
       </c>
-      <c r="F40" s="22" t="inlineStr">
+      <c r="F41" s="22" t="inlineStr">
         <is>
           <t>주임</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="17.25" customHeight="1" s="53" thickTop="1"/>
     <row r="50">
       <c r="C50" s="0" t="n"/>
       <c r="D50" s="0" t="n"/>
@@ -3346,24 +3371,20 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K12" s="22" t="inlineStr">
-        <is>
-          <t>R&amp;D본부</t>
-        </is>
-      </c>
+      <c r="K12" s="22" t="n"/>
       <c r="L12" s="22" t="inlineStr">
         <is>
-          <t>표준모델 개발TF</t>
+          <t>경영기획실</t>
         </is>
       </c>
       <c r="M12" s="22" t="inlineStr">
         <is>
-          <t>최진달미</t>
+          <t>이종원</t>
         </is>
       </c>
       <c r="N12" s="22" t="inlineStr">
         <is>
-          <t>수석연구위원</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
@@ -3414,12 +3435,12 @@
       </c>
       <c r="M13" s="22" t="inlineStr">
         <is>
-          <t>오한솔</t>
+          <t>최진달미</t>
         </is>
       </c>
       <c r="N13" s="22" t="inlineStr">
         <is>
-          <t>연구원</t>
+          <t>수석연구위원</t>
         </is>
       </c>
     </row>
@@ -3465,17 +3486,17 @@
       </c>
       <c r="L14" s="22" t="inlineStr">
         <is>
-          <t>D-LAB 2실</t>
+          <t>표준모델 개발TF</t>
         </is>
       </c>
       <c r="M14" s="22" t="inlineStr">
         <is>
-          <t>최수지</t>
+          <t>오한솔</t>
         </is>
       </c>
       <c r="N14" s="22" t="inlineStr">
         <is>
-          <t>책임연구원</t>
+          <t>연구원</t>
         </is>
       </c>
     </row>
@@ -3503,27 +3524,31 @@
         <v/>
       </c>
       <c r="I15" s="22" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="J15" s="22" t="inlineStr">
         <is>
-          <t>6층</t>
-        </is>
-      </c>
-      <c r="K15" s="22" t="n"/>
+          <t>13층</t>
+        </is>
+      </c>
+      <c r="K15" s="22" t="inlineStr">
+        <is>
+          <t>R&amp;D본부</t>
+        </is>
+      </c>
       <c r="L15" s="22" t="inlineStr">
         <is>
-          <t>신사업개발실</t>
+          <t>D-LAB 2실</t>
         </is>
       </c>
       <c r="M15" s="22" t="inlineStr">
         <is>
-          <t>김태우</t>
+          <t>최수지</t>
         </is>
       </c>
       <c r="N15" s="22" t="inlineStr">
         <is>
-          <t>상무</t>
+          <t>책임연구원</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3560,7 @@
       <c r="E16" s="46" t="n"/>
       <c r="F16" s="12" t="n"/>
       <c r="I16" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16" s="22" t="inlineStr">
         <is>
@@ -3550,12 +3575,12 @@
       </c>
       <c r="M16" s="22" t="inlineStr">
         <is>
-          <t>김순성</t>
+          <t>김태우</t>
         </is>
       </c>
       <c r="N16" s="22" t="inlineStr">
         <is>
-          <t>고문</t>
+          <t>상무</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3604,7 @@
         <v/>
       </c>
       <c r="I17" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J17" s="22" t="inlineStr">
         <is>
@@ -3594,12 +3619,12 @@
       </c>
       <c r="M17" s="22" t="inlineStr">
         <is>
-          <t>박종철</t>
+          <t>김순성</t>
         </is>
       </c>
       <c r="N17" s="22" t="inlineStr">
         <is>
-          <t>이사보</t>
+          <t>고문</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3632,7 @@
       <c r="D18" s="44" t="n"/>
       <c r="E18" s="67" t="n"/>
       <c r="I18" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J18" s="22" t="inlineStr">
         <is>
@@ -3622,12 +3647,12 @@
       </c>
       <c r="M18" s="22" t="inlineStr">
         <is>
-          <t>이정진</t>
+          <t>박종철</t>
         </is>
       </c>
       <c r="N18" s="22" t="inlineStr">
         <is>
-          <t>부장</t>
+          <t>이사보</t>
         </is>
       </c>
     </row>
@@ -3663,31 +3688,27 @@
         </is>
       </c>
       <c r="I19" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J19" s="22" t="inlineStr">
         <is>
-          <t>11층</t>
-        </is>
-      </c>
-      <c r="K19" s="22" t="inlineStr">
-        <is>
-          <t>사업관리본부</t>
-        </is>
-      </c>
+          <t>6층</t>
+        </is>
+      </c>
+      <c r="K19" s="22" t="n"/>
       <c r="L19" s="22" t="inlineStr">
         <is>
-          <t>설계실</t>
+          <t>신사업개발실</t>
         </is>
       </c>
       <c r="M19" s="22" t="inlineStr">
         <is>
-          <t>오진택</t>
+          <t>이정진</t>
         </is>
       </c>
       <c r="N19" s="22" t="inlineStr">
         <is>
-          <t>부사장</t>
+          <t>부장</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3740,7 @@
         <v/>
       </c>
       <c r="I20" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="22" t="inlineStr">
         <is>
@@ -3738,12 +3759,12 @@
       </c>
       <c r="M20" s="22" t="inlineStr">
         <is>
-          <t>최우제</t>
+          <t>오진택</t>
         </is>
       </c>
       <c r="N20" s="22" t="inlineStr">
         <is>
-          <t>상무</t>
+          <t>부사장</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3796,7 @@
         <v/>
       </c>
       <c r="I21" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J21" s="22" t="inlineStr">
         <is>
@@ -3794,12 +3815,12 @@
       </c>
       <c r="M21" s="22" t="inlineStr">
         <is>
-          <t>김채영</t>
+          <t>최우제</t>
         </is>
       </c>
       <c r="N21" s="22" t="inlineStr">
         <is>
-          <t>이사보</t>
+          <t>상무</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3852,7 @@
         <v/>
       </c>
       <c r="I22" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J22" s="22" t="inlineStr">
         <is>
@@ -3850,12 +3871,12 @@
       </c>
       <c r="M22" s="22" t="inlineStr">
         <is>
-          <t>김태은</t>
+          <t>김채영</t>
         </is>
       </c>
       <c r="N22" s="22" t="inlineStr">
         <is>
-          <t>과장</t>
+          <t>이사보</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3908,7 @@
         <v/>
       </c>
       <c r="I23" s="22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J23" s="22" t="inlineStr">
         <is>
@@ -3906,12 +3927,12 @@
       </c>
       <c r="M23" s="22" t="inlineStr">
         <is>
-          <t>김민호</t>
+          <t>김태은</t>
         </is>
       </c>
       <c r="N23" s="22" t="inlineStr">
         <is>
-          <t>대리</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3960,7 @@
         <v/>
       </c>
       <c r="I24" s="22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J24" s="22" t="inlineStr">
         <is>
@@ -3958,12 +3979,12 @@
       </c>
       <c r="M24" s="22" t="inlineStr">
         <is>
-          <t>이수영</t>
+          <t>김민호</t>
         </is>
       </c>
       <c r="N24" s="22" t="inlineStr">
         <is>
-          <t>주임</t>
+          <t>대리</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3996,7 @@
       <c r="E25" s="46" t="n"/>
       <c r="F25" s="12" t="n"/>
       <c r="I25" s="22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J25" s="22" t="inlineStr">
         <is>
@@ -3994,12 +4015,12 @@
       </c>
       <c r="M25" s="22" t="inlineStr">
         <is>
-          <t>최수용</t>
+          <t>이수영</t>
         </is>
       </c>
       <c r="N25" s="22" t="inlineStr">
         <is>
-          <t>사원</t>
+          <t>주임</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4032,7 @@
       <c r="E26" s="46" t="n"/>
       <c r="F26" s="12" t="n"/>
       <c r="I26" s="22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J26" s="22" t="inlineStr">
         <is>
@@ -4025,17 +4046,17 @@
       </c>
       <c r="L26" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>설계실</t>
         </is>
       </c>
       <c r="M26" s="22" t="inlineStr">
         <is>
-          <t>김동우</t>
+          <t>최수용</t>
         </is>
       </c>
       <c r="N26" s="22" t="inlineStr">
         <is>
-          <t>부사장</t>
+          <t>사원</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4068,7 @@
       <c r="E27" s="46" t="n"/>
       <c r="F27" s="12" t="n"/>
       <c r="I27" s="22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J27" s="22" t="inlineStr">
         <is>
@@ -4066,12 +4087,12 @@
       </c>
       <c r="M27" s="22" t="inlineStr">
         <is>
-          <t>이성규</t>
+          <t>김동우</t>
         </is>
       </c>
       <c r="N27" s="22" t="inlineStr">
         <is>
-          <t>차장</t>
+          <t>부사장</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4104,7 @@
       <c r="E28" s="46" t="n"/>
       <c r="F28" s="12" t="n"/>
       <c r="I28" s="22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J28" s="22" t="inlineStr">
         <is>
@@ -4102,7 +4123,7 @@
       </c>
       <c r="M28" s="22" t="inlineStr">
         <is>
-          <t>이강호</t>
+          <t>이성규</t>
         </is>
       </c>
       <c r="N28" s="22" t="inlineStr">
@@ -4119,7 +4140,7 @@
       <c r="E29" s="46" t="n"/>
       <c r="F29" s="12" t="n"/>
       <c r="I29" s="22" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J29" s="22" t="inlineStr">
         <is>
@@ -4138,12 +4159,12 @@
       </c>
       <c r="M29" s="22" t="inlineStr">
         <is>
-          <t>김동규</t>
+          <t>이강호</t>
         </is>
       </c>
       <c r="N29" s="22" t="inlineStr">
         <is>
-          <t>부장</t>
+          <t>차장</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4176,7 @@
       <c r="E30" s="46" t="n"/>
       <c r="F30" s="12" t="n"/>
       <c r="I30" s="22" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J30" s="22" t="inlineStr">
         <is>
@@ -4169,17 +4190,17 @@
       </c>
       <c r="L30" s="22" t="inlineStr">
         <is>
-          <t>사업관리1실</t>
+          <t>사업관리본부</t>
         </is>
       </c>
       <c r="M30" s="22" t="inlineStr">
         <is>
-          <t>김승현</t>
+          <t>김동규</t>
         </is>
       </c>
       <c r="N30" s="22" t="inlineStr">
         <is>
-          <t>상무</t>
+          <t>부장</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4212,7 @@
       <c r="E31" s="46" t="n"/>
       <c r="F31" s="12" t="n"/>
       <c r="I31" s="22" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J31" s="22" t="inlineStr">
         <is>
@@ -4210,12 +4231,12 @@
       </c>
       <c r="M31" s="22" t="inlineStr">
         <is>
-          <t>조지은</t>
+          <t>김승현</t>
         </is>
       </c>
       <c r="N31" s="22" t="inlineStr">
         <is>
-          <t>이사보</t>
+          <t>상무</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4248,7 @@
       <c r="E32" s="46" t="n"/>
       <c r="F32" s="12" t="n"/>
       <c r="I32" s="22" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J32" s="22" t="inlineStr">
         <is>
@@ -4246,12 +4267,12 @@
       </c>
       <c r="M32" s="22" t="inlineStr">
         <is>
-          <t>이예솔</t>
+          <t>조지은</t>
         </is>
       </c>
       <c r="N32" s="22" t="inlineStr">
         <is>
-          <t>과장</t>
+          <t>이사보</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4284,7 @@
       <c r="E33" s="46" t="n"/>
       <c r="F33" s="12" t="n"/>
       <c r="I33" s="22" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J33" s="22" t="inlineStr">
         <is>
@@ -4282,7 +4303,7 @@
       </c>
       <c r="M33" s="22" t="inlineStr">
         <is>
-          <t>류승호</t>
+          <t>이예솔</t>
         </is>
       </c>
       <c r="N33" s="22" t="inlineStr">
@@ -4299,7 +4320,7 @@
       <c r="E34" s="46" t="n"/>
       <c r="F34" s="12" t="n"/>
       <c r="I34" s="22" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J34" s="22" t="inlineStr">
         <is>
@@ -4313,17 +4334,17 @@
       </c>
       <c r="L34" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>사업관리1실</t>
         </is>
       </c>
       <c r="M34" s="22" t="inlineStr">
         <is>
-          <t>주현철</t>
+          <t>류승호</t>
         </is>
       </c>
       <c r="N34" s="22" t="inlineStr">
         <is>
-          <t>상무</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4356,7 @@
       <c r="E35" s="46" t="n"/>
       <c r="F35" s="12" t="n"/>
       <c r="I35" s="22" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J35" s="22" t="inlineStr">
         <is>
@@ -4354,12 +4375,12 @@
       </c>
       <c r="M35" s="22" t="inlineStr">
         <is>
-          <t>이완구</t>
+          <t>주현철</t>
         </is>
       </c>
       <c r="N35" s="22" t="inlineStr">
         <is>
-          <t>이사보</t>
+          <t>상무</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4392,7 @@
       <c r="E36" s="46" t="n"/>
       <c r="F36" s="12" t="n"/>
       <c r="I36" s="22" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J36" s="22" t="inlineStr">
         <is>
@@ -4390,12 +4411,12 @@
       </c>
       <c r="M36" s="22" t="inlineStr">
         <is>
-          <t>황진욱</t>
+          <t>이완구</t>
         </is>
       </c>
       <c r="N36" s="22" t="inlineStr">
         <is>
-          <t>대리</t>
+          <t>이사보</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4428,7 @@
       <c r="E37" s="46" t="n"/>
       <c r="F37" s="12" t="n"/>
       <c r="I37" s="22" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J37" s="22" t="inlineStr">
         <is>
@@ -4426,12 +4447,12 @@
       </c>
       <c r="M37" s="22" t="inlineStr">
         <is>
-          <t>문광정</t>
+          <t>황진욱</t>
         </is>
       </c>
       <c r="N37" s="22" t="inlineStr">
         <is>
-          <t>부장</t>
+          <t>대리</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4464,7 @@
       <c r="E38" s="46" t="n"/>
       <c r="F38" s="12" t="n"/>
       <c r="I38" s="22" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J38" s="22" t="inlineStr">
         <is>
@@ -4462,12 +4483,12 @@
       </c>
       <c r="M38" s="22" t="inlineStr">
         <is>
-          <t>정연석</t>
+          <t>문광정</t>
         </is>
       </c>
       <c r="N38" s="22" t="inlineStr">
         <is>
-          <t>대리</t>
+          <t>부장</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4500,7 @@
       <c r="E39" s="46" t="n"/>
       <c r="F39" s="12" t="n"/>
       <c r="I39" s="22" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J39" s="22" t="inlineStr">
         <is>
@@ -4498,7 +4519,7 @@
       </c>
       <c r="M39" s="22" t="inlineStr">
         <is>
-          <t>김진규</t>
+          <t>정연석</t>
         </is>
       </c>
       <c r="N39" s="22" t="inlineStr">
@@ -4515,7 +4536,7 @@
       <c r="E40" s="12" t="n"/>
       <c r="F40" s="12" t="n"/>
       <c r="I40" s="22" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J40" s="22" t="inlineStr">
         <is>
@@ -4534,12 +4555,12 @@
       </c>
       <c r="M40" s="22" t="inlineStr">
         <is>
-          <t>연지현</t>
+          <t>김진규</t>
         </is>
       </c>
       <c r="N40" s="22" t="inlineStr">
         <is>
-          <t>주임</t>
+          <t>대리</t>
         </is>
       </c>
     </row>
@@ -4550,6 +4571,34 @@
       <c r="D41" s="12" t="n"/>
       <c r="E41" s="12" t="n"/>
       <c r="F41" s="12" t="n"/>
+      <c r="I41" s="22" t="n">
+        <v>22</v>
+      </c>
+      <c r="J41" s="22" t="inlineStr">
+        <is>
+          <t>11층</t>
+        </is>
+      </c>
+      <c r="K41" s="22" t="inlineStr">
+        <is>
+          <t>사업관리본부</t>
+        </is>
+      </c>
+      <c r="L41" s="22" t="inlineStr">
+        <is>
+          <t>사업관리2실</t>
+        </is>
+      </c>
+      <c r="M41" s="22" t="inlineStr">
+        <is>
+          <t>연지현</t>
+        </is>
+      </c>
+      <c r="N41" s="22" t="inlineStr">
+        <is>
+          <t>주임</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="12" t="n"/>

</xml_diff>

<commit_message>
Split October electricity allocation by team
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FM2YJqCagBbEuBH1oLpGAS
</commit_message>
<xml_diff>
--- a/out/전기세_지출결의서_26.10.xlsx
+++ b/out/전기세_지출결의서_26.10.xlsx
@@ -787,12 +787,12 @@
         <t>단수차이 자동 조정(총액-다른 부서 합)</t>
       </text>
     </comment>
-    <comment ref="D14" authorId="0" shapeId="0">
+    <comment ref="D18" authorId="0" shapeId="0">
       <text>
         <t>단수차이 자동 조정(총액-다른 부서 합)</t>
       </text>
     </comment>
-    <comment ref="D23" authorId="0" shapeId="0">
+    <comment ref="D29" authorId="0" shapeId="0">
       <text>
         <t>단수차이 자동 조정(총액-다른 부서 합)</t>
       </text>
@@ -1210,20 +1210,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C4" s="22" t="n"/>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D4" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획1팀</t>
         </is>
       </c>
       <c r="E4" s="22" t="inlineStr">
         <is>
-          <t>조승제</t>
+          <t>이경태</t>
         </is>
       </c>
       <c r="F4" s="22" t="inlineStr">
         <is>
-          <t>부장</t>
+          <t>차장</t>
         </is>
       </c>
     </row>
@@ -1236,10 +1240,14 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C5" s="22" t="n"/>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획1팀</t>
         </is>
       </c>
       <c r="E5" s="22" t="inlineStr">
@@ -1262,15 +1270,19 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C6" s="22" t="n"/>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D6" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획1팀</t>
         </is>
       </c>
       <c r="E6" s="22" t="inlineStr">
         <is>
-          <t>강지혜</t>
+          <t>이황</t>
         </is>
       </c>
       <c r="F6" s="22" t="inlineStr">
@@ -1288,20 +1300,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C7" s="22" t="n"/>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획1팀</t>
         </is>
       </c>
       <c r="E7" s="22" t="inlineStr">
         <is>
-          <t>이경태</t>
+          <t>이종원</t>
         </is>
       </c>
       <c r="F7" s="22" t="inlineStr">
         <is>
-          <t>차장</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
@@ -1314,20 +1330,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n"/>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="E8" s="22" t="inlineStr">
         <is>
-          <t>최경천</t>
+          <t>조승제</t>
         </is>
       </c>
       <c r="F8" s="22" t="inlineStr">
         <is>
-          <t>차장</t>
+          <t>부장</t>
         </is>
       </c>
     </row>
@@ -1340,15 +1360,19 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n"/>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="E9" s="22" t="inlineStr">
         <is>
-          <t>이재선</t>
+          <t>최경천</t>
         </is>
       </c>
       <c r="F9" s="22" t="inlineStr">
@@ -1366,20 +1390,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C10" s="22" t="n"/>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="E10" s="22" t="inlineStr">
         <is>
-          <t>이황</t>
+          <t>이재선</t>
         </is>
       </c>
       <c r="F10" s="22" t="inlineStr">
         <is>
-          <t>과장</t>
+          <t>차장</t>
         </is>
       </c>
     </row>
@@ -1392,20 +1420,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C11" s="22" t="n"/>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="E11" s="22" t="inlineStr">
         <is>
-          <t>강소영</t>
+          <t>강지혜</t>
         </is>
       </c>
       <c r="F11" s="22" t="inlineStr">
         <is>
-          <t>대리</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
@@ -1418,20 +1450,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="C12" s="22" t="n"/>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="E12" s="22" t="inlineStr">
         <is>
-          <t>이종원</t>
+          <t>강소영</t>
         </is>
       </c>
       <c r="F12" s="22" t="inlineStr">
         <is>
-          <t>과장</t>
+          <t>대리</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1921,7 @@
       </c>
       <c r="D28" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업기획팀</t>
         </is>
       </c>
       <c r="E28" s="22" t="inlineStr">
@@ -1915,7 +1951,7 @@
       </c>
       <c r="D29" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업지원팀</t>
         </is>
       </c>
       <c r="E29" s="22" t="inlineStr">
@@ -1945,7 +1981,7 @@
       </c>
       <c r="D30" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업지원팀</t>
         </is>
       </c>
       <c r="E30" s="22" t="inlineStr">
@@ -2120,12 +2156,12 @@
       </c>
       <c r="C36" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="D36" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>사업관리팀</t>
         </is>
       </c>
       <c r="E36" s="22" t="inlineStr">
@@ -2150,12 +2186,12 @@
       </c>
       <c r="C37" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="D37" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>사업관리팀</t>
         </is>
       </c>
       <c r="E37" s="22" t="inlineStr">
@@ -2180,12 +2216,12 @@
       </c>
       <c r="C38" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="D38" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>영업기획팀</t>
         </is>
       </c>
       <c r="E38" s="22" t="inlineStr">
@@ -2211,12 +2247,12 @@
       </c>
       <c r="C39" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="D39" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>영업기획팀</t>
         </is>
       </c>
       <c r="E39" s="22" t="inlineStr">
@@ -2242,12 +2278,12 @@
       </c>
       <c r="C40" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="D40" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>영업기획팀</t>
         </is>
       </c>
       <c r="E40" s="22" t="inlineStr">
@@ -2272,12 +2308,12 @@
       </c>
       <c r="C41" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="D41" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>영업기획팀</t>
         </is>
       </c>
       <c r="E41" s="22" t="inlineStr">
@@ -3007,20 +3043,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K4" s="22" t="n"/>
+      <c r="K4" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L4" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획1팀</t>
         </is>
       </c>
       <c r="M4" s="22" t="inlineStr">
         <is>
-          <t>조승제</t>
+          <t>이경태</t>
         </is>
       </c>
       <c r="N4" s="22" t="inlineStr">
         <is>
-          <t>부장</t>
+          <t>차장</t>
         </is>
       </c>
     </row>
@@ -3059,10 +3099,14 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K5" s="22" t="n"/>
+      <c r="K5" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L5" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획1팀</t>
         </is>
       </c>
       <c r="M5" s="22" t="inlineStr">
@@ -3107,15 +3151,19 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K6" s="22" t="n"/>
+      <c r="K6" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L6" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획1팀</t>
         </is>
       </c>
       <c r="M6" s="22" t="inlineStr">
         <is>
-          <t>강지혜</t>
+          <t>이황</t>
         </is>
       </c>
       <c r="N6" s="22" t="inlineStr">
@@ -3139,20 +3187,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K7" s="22" t="n"/>
+      <c r="K7" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L7" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획1팀</t>
         </is>
       </c>
       <c r="M7" s="22" t="inlineStr">
         <is>
-          <t>이경태</t>
+          <t>이종원</t>
         </is>
       </c>
       <c r="N7" s="22" t="inlineStr">
         <is>
-          <t>차장</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
@@ -3183,20 +3235,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K8" s="22" t="n"/>
+      <c r="K8" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L8" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="M8" s="22" t="inlineStr">
         <is>
-          <t>최경천</t>
+          <t>조승제</t>
         </is>
       </c>
       <c r="N8" s="22" t="inlineStr">
         <is>
-          <t>차장</t>
+          <t>부장</t>
         </is>
       </c>
     </row>
@@ -3211,15 +3267,19 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K9" s="22" t="n"/>
+      <c r="K9" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L9" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="M9" s="22" t="inlineStr">
         <is>
-          <t>이재선</t>
+          <t>최경천</t>
         </is>
       </c>
       <c r="N9" s="22" t="inlineStr">
@@ -3267,20 +3327,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K10" s="22" t="n"/>
+      <c r="K10" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L10" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="M10" s="22" t="inlineStr">
         <is>
-          <t>이황</t>
+          <t>이재선</t>
         </is>
       </c>
       <c r="N10" s="22" t="inlineStr">
         <is>
-          <t>과장</t>
+          <t>차장</t>
         </is>
       </c>
     </row>
@@ -3300,11 +3364,11 @@
         <v/>
       </c>
       <c r="D11" s="75">
-        <f>ROUND($D$8/$C$15*C11,0)</f>
+        <f>ROUND($D$8/$C$19*C11,0)</f>
         <v/>
       </c>
       <c r="E11" s="75">
-        <f>ROUND($E$8/$C$15*C11,0)</f>
+        <f>ROUND($E$8/$C$19*C11,0)</f>
         <v/>
       </c>
       <c r="F11" s="76">
@@ -3319,20 +3383,24 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K11" s="22" t="n"/>
+      <c r="K11" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L11" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="M11" s="22" t="inlineStr">
         <is>
-          <t>강소영</t>
+          <t>강지혜</t>
         </is>
       </c>
       <c r="N11" s="22" t="inlineStr">
         <is>
-          <t>대리</t>
+          <t>과장</t>
         </is>
       </c>
     </row>
@@ -3352,11 +3420,11 @@
         <v/>
       </c>
       <c r="D12" s="75">
-        <f>ROUND($D$8/$C$15*C12,0)</f>
+        <f>ROUND($D$8/$C$19*C12,0)</f>
         <v/>
       </c>
       <c r="E12" s="75">
-        <f>ROUND($E$8/$C$15*C12,0)</f>
+        <f>ROUND($E$8/$C$19*C12,0)</f>
         <v/>
       </c>
       <c r="F12" s="76">
@@ -3371,27 +3439,31 @@
           <t>13층</t>
         </is>
       </c>
-      <c r="K12" s="22" t="n"/>
+      <c r="K12" s="22" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
       <c r="L12" s="22" t="inlineStr">
         <is>
-          <t>경영기획실</t>
+          <t>경영기획2팀</t>
         </is>
       </c>
       <c r="M12" s="22" t="inlineStr">
         <is>
-          <t>이종원</t>
+          <t>강소영</t>
         </is>
       </c>
       <c r="N12" s="22" t="inlineStr">
         <is>
-          <t>과장</t>
+          <t>대리</t>
         </is>
       </c>
     </row>
     <row r="13" ht="17.25" customHeight="1" s="53">
       <c r="A13" s="72" t="inlineStr">
         <is>
-          <t>사업관리1실</t>
+          <t>사업기획팀</t>
         </is>
       </c>
       <c r="B13" s="73" t="inlineStr">
@@ -3400,15 +3472,15 @@
         </is>
       </c>
       <c r="C13" s="74">
-        <f>COUNTIF(L:L,"사업관리1실")</f>
+        <f>COUNTIF(L:L,"사업기획팀")</f>
         <v/>
       </c>
       <c r="D13" s="75">
-        <f>ROUND($D$8/$C$15*C13,0)</f>
+        <f>ROUND($D$8/$C$19*C13,0)</f>
         <v/>
       </c>
       <c r="E13" s="75">
-        <f>ROUND($E$8/$C$15*C13,0)</f>
+        <f>ROUND($E$8/$C$19*C13,0)</f>
         <v/>
       </c>
       <c r="F13" s="76">
@@ -3447,7 +3519,7 @@
     <row r="14">
       <c r="A14" s="72" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>사업지원팀</t>
         </is>
       </c>
       <c r="B14" s="73" t="inlineStr">
@@ -3456,15 +3528,15 @@
         </is>
       </c>
       <c r="C14" s="74">
-        <f>COUNTIF(L:L,"사업관리2실")</f>
+        <f>COUNTIF(L:L,"사업지원팀")</f>
         <v/>
       </c>
       <c r="D14" s="75">
-        <f>$D$8-SUM(D11:D13)</f>
+        <f>ROUND($D$8/$C$19*C14,0)</f>
         <v/>
       </c>
       <c r="E14" s="75">
-        <f>$E$8-SUM(E11:E13)</f>
+        <f>ROUND($E$8/$C$19*C14,0)</f>
         <v/>
       </c>
       <c r="F14" s="76">
@@ -3501,26 +3573,30 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="68" t="inlineStr">
-        <is>
-          <t>총합</t>
-        </is>
-      </c>
-      <c r="B15" s="69" t="n"/>
-      <c r="C15" s="70">
-        <f>SUM(C11:C14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="77">
-        <f>SUM(D11:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="77">
-        <f>SUM(E11:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="78">
-        <f>SUM(F11:F14)</f>
+      <c r="A15" s="72" t="inlineStr">
+        <is>
+          <t>사업관리1실</t>
+        </is>
+      </c>
+      <c r="B15" s="73" t="inlineStr">
+        <is>
+          <t>판관</t>
+        </is>
+      </c>
+      <c r="C15" s="74">
+        <f>COUNTIF(L:L,"사업관리1실")</f>
+        <v/>
+      </c>
+      <c r="D15" s="75">
+        <f>ROUND($D$8/$C$19*C15,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="75">
+        <f>ROUND($E$8/$C$19*C15,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="76">
+        <f>D15+E15</f>
         <v/>
       </c>
       <c r="I15" s="22" t="n">
@@ -3553,12 +3629,32 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="46" t="n"/>
-      <c r="F16" s="12" t="n"/>
+      <c r="A16" s="72" t="inlineStr">
+        <is>
+          <t>사업관리2실</t>
+        </is>
+      </c>
+      <c r="B16" s="73" t="inlineStr">
+        <is>
+          <t>판관</t>
+        </is>
+      </c>
+      <c r="C16" s="74">
+        <f>COUNTIF(L:L,"사업관리2실")</f>
+        <v/>
+      </c>
+      <c r="D16" s="75">
+        <f>ROUND($D$8/$C$19*C16,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="75">
+        <f>ROUND($E$8/$C$19*C16,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="76">
+        <f>D16+E16</f>
+        <v/>
+      </c>
       <c r="I16" s="22" t="n">
         <v>1</v>
       </c>
@@ -3585,21 +3681,29 @@
       </c>
     </row>
     <row r="17" ht="17.25" customHeight="1" s="53" thickBot="1">
-      <c r="A17" s="64" t="inlineStr">
-        <is>
-          <t>전기료 총액(13층)</t>
-        </is>
-      </c>
-      <c r="B17" s="55" t="n"/>
-      <c r="C17" s="56" t="n"/>
-      <c r="D17" s="79">
-        <f>308764+8330</f>
-        <v/>
-      </c>
-      <c r="E17" s="79" t="n">
-        <v>30876</v>
-      </c>
-      <c r="F17" s="66">
+      <c r="A17" s="72" t="inlineStr">
+        <is>
+          <t>사업관리팀</t>
+        </is>
+      </c>
+      <c r="B17" s="73" t="inlineStr">
+        <is>
+          <t>판관</t>
+        </is>
+      </c>
+      <c r="C17" s="74">
+        <f>COUNTIF(L:L,"사업관리팀")</f>
+        <v/>
+      </c>
+      <c r="D17" s="75">
+        <f>ROUND($D$8/$C$19*C17,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="75">
+        <f>ROUND($E$8/$C$19*C17,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="76">
         <f>D17+E17</f>
         <v/>
       </c>
@@ -3629,8 +3733,32 @@
       </c>
     </row>
     <row r="18" ht="17.25" customHeight="1" s="53" thickBot="1">
-      <c r="D18" s="44" t="n"/>
-      <c r="E18" s="67" t="n"/>
+      <c r="A18" s="72" t="inlineStr">
+        <is>
+          <t>영업기획팀</t>
+        </is>
+      </c>
+      <c r="B18" s="73" t="inlineStr">
+        <is>
+          <t>판관</t>
+        </is>
+      </c>
+      <c r="C18" s="74">
+        <f>COUNTIF(L:L,"영업기획팀")</f>
+        <v/>
+      </c>
+      <c r="D18" s="75">
+        <f>$D$8-SUM(D11:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="75">
+        <f>$E$8-SUM(E11:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="76">
+        <f>D18+E18</f>
+        <v/>
+      </c>
       <c r="I18" s="22" t="n">
         <v>3</v>
       </c>
@@ -3659,33 +3787,25 @@
     <row r="19" ht="17.25" customHeight="1" s="53" thickBot="1">
       <c r="A19" s="68" t="inlineStr">
         <is>
-          <t>부서</t>
-        </is>
-      </c>
-      <c r="B19" s="69" t="inlineStr">
-        <is>
-          <t>계정</t>
-        </is>
-      </c>
-      <c r="C19" s="70" t="inlineStr">
-        <is>
-          <t>인원</t>
-        </is>
-      </c>
-      <c r="D19" s="28" t="inlineStr">
-        <is>
-          <t>공급가</t>
-        </is>
-      </c>
-      <c r="E19" s="71" t="inlineStr">
-        <is>
-          <t>부가세</t>
-        </is>
-      </c>
-      <c r="F19" s="30" t="inlineStr">
-        <is>
-          <t>합계</t>
-        </is>
+          <t>총합</t>
+        </is>
+      </c>
+      <c r="B19" s="69" t="n"/>
+      <c r="C19" s="70">
+        <f>SUM(C11:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="77">
+        <f>SUM(D11:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="77">
+        <f>SUM(E11:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="78">
+        <f>SUM(F11:F18)</f>
+        <v/>
       </c>
       <c r="I19" s="22" t="n">
         <v>4</v>
@@ -3713,32 +3833,12 @@
       </c>
     </row>
     <row r="20" ht="17.25" customHeight="1" s="53" thickBot="1">
-      <c r="A20" s="72" t="inlineStr">
-        <is>
-          <t>경영기획실</t>
-        </is>
-      </c>
-      <c r="B20" s="73" t="inlineStr">
-        <is>
-          <t>판관</t>
-        </is>
-      </c>
-      <c r="C20" s="74">
-        <f>COUNTIF(L:L,"경영기획실")</f>
-        <v/>
-      </c>
-      <c r="D20" s="75">
-        <f>ROUND($D$17/$C$24*C20,0)</f>
-        <v/>
-      </c>
-      <c r="E20" s="75">
-        <f>ROUND($E$17/$C$24*C20,0)</f>
-        <v/>
-      </c>
-      <c r="F20" s="76">
-        <f>D20+E20</f>
-        <v/>
-      </c>
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="46" t="n"/>
+      <c r="F20" s="12" t="n"/>
       <c r="I20" s="22" t="n">
         <v>1</v>
       </c>
@@ -3769,29 +3869,21 @@
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" s="53" thickBot="1">
-      <c r="A21" s="72" t="inlineStr">
-        <is>
-          <t>R&amp;D본부</t>
-        </is>
-      </c>
-      <c r="B21" s="73" t="inlineStr">
-        <is>
-          <t>연구</t>
-        </is>
-      </c>
-      <c r="C21" s="74">
-        <f>COUNTIF(L:L,"R&amp;D본부")</f>
-        <v/>
-      </c>
-      <c r="D21" s="75">
-        <f>ROUND($D$17/$C$24*C21,0)</f>
-        <v/>
-      </c>
-      <c r="E21" s="75">
-        <f>ROUND($E$17/$C$24*C21,0)</f>
-        <v/>
-      </c>
-      <c r="F21" s="76">
+      <c r="A21" s="64" t="inlineStr">
+        <is>
+          <t>전기료 총액(13층)</t>
+        </is>
+      </c>
+      <c r="B21" s="55" t="n"/>
+      <c r="C21" s="56" t="n"/>
+      <c r="D21" s="79">
+        <f>308764+8330</f>
+        <v/>
+      </c>
+      <c r="E21" s="79" t="n">
+        <v>30876</v>
+      </c>
+      <c r="F21" s="66">
         <f>D21+E21</f>
         <v/>
       </c>
@@ -3825,32 +3917,8 @@
       </c>
     </row>
     <row r="22" ht="17.25" customHeight="1" s="53" thickBot="1">
-      <c r="A22" s="72" t="inlineStr">
-        <is>
-          <t>표준모델 개발TF</t>
-        </is>
-      </c>
-      <c r="B22" s="73" t="inlineStr">
-        <is>
-          <t>연구</t>
-        </is>
-      </c>
-      <c r="C22" s="74">
-        <f>COUNTIF(L:L,"표준모델 개발TF")</f>
-        <v/>
-      </c>
-      <c r="D22" s="75">
-        <f>ROUND($D$17/$C$24*C22,0)</f>
-        <v/>
-      </c>
-      <c r="E22" s="75">
-        <f>ROUND($E$17/$C$24*C22,0)</f>
-        <v/>
-      </c>
-      <c r="F22" s="76">
-        <f>D22+E22</f>
-        <v/>
-      </c>
+      <c r="D22" s="44" t="n"/>
+      <c r="E22" s="67" t="n"/>
       <c r="I22" s="22" t="n">
         <v>3</v>
       </c>
@@ -3881,31 +3949,35 @@
       </c>
     </row>
     <row r="23" ht="17.25" customHeight="1" s="53">
-      <c r="A23" s="72" t="inlineStr">
-        <is>
-          <t>D-LAB 2실</t>
-        </is>
-      </c>
-      <c r="B23" s="73" t="inlineStr">
-        <is>
-          <t>연구</t>
-        </is>
-      </c>
-      <c r="C23" s="74">
-        <f>COUNTIF(L:L,"D-LAB 2실")</f>
-        <v/>
-      </c>
-      <c r="D23" s="75">
-        <f>$D$17-SUM(D20:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="75">
-        <f>$E$17-SUM(E20:E22)</f>
-        <v/>
-      </c>
-      <c r="F23" s="76">
-        <f>D23+E23</f>
-        <v/>
+      <c r="A23" s="68" t="inlineStr">
+        <is>
+          <t>부서</t>
+        </is>
+      </c>
+      <c r="B23" s="69" t="inlineStr">
+        <is>
+          <t>계정</t>
+        </is>
+      </c>
+      <c r="C23" s="70" t="inlineStr">
+        <is>
+          <t>인원</t>
+        </is>
+      </c>
+      <c r="D23" s="28" t="inlineStr">
+        <is>
+          <t>공급가</t>
+        </is>
+      </c>
+      <c r="E23" s="71" t="inlineStr">
+        <is>
+          <t>부가세</t>
+        </is>
+      </c>
+      <c r="F23" s="30" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
       </c>
       <c r="I23" s="22" t="n">
         <v>4</v>
@@ -3937,26 +4009,30 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="68" t="inlineStr">
-        <is>
-          <t>총합</t>
-        </is>
-      </c>
-      <c r="B24" s="69" t="n"/>
-      <c r="C24" s="70">
-        <f>SUM(C20:C23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="77">
-        <f>SUM(D20:D23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="77">
-        <f>SUM(E20:E23)</f>
-        <v/>
-      </c>
-      <c r="F24" s="78">
-        <f>SUM(F20:F23)</f>
+      <c r="A24" s="72" t="inlineStr">
+        <is>
+          <t>경영기획실</t>
+        </is>
+      </c>
+      <c r="B24" s="73" t="inlineStr">
+        <is>
+          <t>판관</t>
+        </is>
+      </c>
+      <c r="C24" s="74">
+        <f>COUNTIF(L:L,"경영기획실")</f>
+        <v/>
+      </c>
+      <c r="D24" s="75">
+        <f>ROUND($D$21/$C$30*C24,0)</f>
+        <v/>
+      </c>
+      <c r="E24" s="75">
+        <f>ROUND($E$21/$C$30*C24,0)</f>
+        <v/>
+      </c>
+      <c r="F24" s="76">
+        <f>D24+E24</f>
         <v/>
       </c>
       <c r="I24" s="22" t="n">
@@ -3989,12 +4065,32 @@
       </c>
     </row>
     <row r="25" ht="17.25" customHeight="1" s="53" thickBot="1">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="12" t="n"/>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="46" t="n"/>
-      <c r="F25" s="12" t="n"/>
+      <c r="A25" s="72" t="inlineStr">
+        <is>
+          <t>경영기획1팀</t>
+        </is>
+      </c>
+      <c r="B25" s="73" t="inlineStr">
+        <is>
+          <t>판관</t>
+        </is>
+      </c>
+      <c r="C25" s="74">
+        <f>COUNTIF(L:L,"경영기획1팀")</f>
+        <v/>
+      </c>
+      <c r="D25" s="75">
+        <f>ROUND($D$21/$C$30*C25,0)</f>
+        <v/>
+      </c>
+      <c r="E25" s="75">
+        <f>ROUND($E$21/$C$30*C25,0)</f>
+        <v/>
+      </c>
+      <c r="F25" s="76">
+        <f>D25+E25</f>
+        <v/>
+      </c>
       <c r="I25" s="22" t="n">
         <v>6</v>
       </c>
@@ -4025,12 +4121,32 @@
       </c>
     </row>
     <row r="26" ht="17.25" customHeight="1" s="53" thickBot="1" thickTop="1">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="46" t="n"/>
-      <c r="F26" s="12" t="n"/>
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>경영기획2팀</t>
+        </is>
+      </c>
+      <c r="B26" s="73" t="inlineStr">
+        <is>
+          <t>판관</t>
+        </is>
+      </c>
+      <c r="C26" s="74">
+        <f>COUNTIF(L:L,"경영기획2팀")</f>
+        <v/>
+      </c>
+      <c r="D26" s="75">
+        <f>ROUND($D$21/$C$30*C26,0)</f>
+        <v/>
+      </c>
+      <c r="E26" s="75">
+        <f>ROUND($E$21/$C$30*C26,0)</f>
+        <v/>
+      </c>
+      <c r="F26" s="76">
+        <f>D26+E26</f>
+        <v/>
+      </c>
       <c r="I26" s="22" t="n">
         <v>7</v>
       </c>
@@ -4061,12 +4177,32 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="53">
-      <c r="A27" s="12" t="n"/>
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="46" t="n"/>
-      <c r="F27" s="12" t="n"/>
+      <c r="A27" s="72" t="inlineStr">
+        <is>
+          <t>R&amp;D본부</t>
+        </is>
+      </c>
+      <c r="B27" s="73" t="inlineStr">
+        <is>
+          <t>연구</t>
+        </is>
+      </c>
+      <c r="C27" s="74">
+        <f>COUNTIF(L:L,"R&amp;D본부")</f>
+        <v/>
+      </c>
+      <c r="D27" s="75">
+        <f>ROUND($D$21/$C$30*C27,0)</f>
+        <v/>
+      </c>
+      <c r="E27" s="75">
+        <f>ROUND($E$21/$C$30*C27,0)</f>
+        <v/>
+      </c>
+      <c r="F27" s="76">
+        <f>D27+E27</f>
+        <v/>
+      </c>
       <c r="I27" s="22" t="n">
         <v>8</v>
       </c>
@@ -4097,12 +4233,32 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="46" t="n"/>
-      <c r="F28" s="12" t="n"/>
+      <c r="A28" s="72" t="inlineStr">
+        <is>
+          <t>표준모델 개발TF</t>
+        </is>
+      </c>
+      <c r="B28" s="73" t="inlineStr">
+        <is>
+          <t>연구</t>
+        </is>
+      </c>
+      <c r="C28" s="74">
+        <f>COUNTIF(L:L,"표준모델 개발TF")</f>
+        <v/>
+      </c>
+      <c r="D28" s="75">
+        <f>ROUND($D$21/$C$30*C28,0)</f>
+        <v/>
+      </c>
+      <c r="E28" s="75">
+        <f>ROUND($E$21/$C$30*C28,0)</f>
+        <v/>
+      </c>
+      <c r="F28" s="76">
+        <f>D28+E28</f>
+        <v/>
+      </c>
       <c r="I28" s="22" t="n">
         <v>9</v>
       </c>
@@ -4118,7 +4274,7 @@
       </c>
       <c r="L28" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업기획팀</t>
         </is>
       </c>
       <c r="M28" s="22" t="inlineStr">
@@ -4133,12 +4289,32 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="46" t="n"/>
-      <c r="F29" s="12" t="n"/>
+      <c r="A29" s="72" t="inlineStr">
+        <is>
+          <t>D-LAB 2실</t>
+        </is>
+      </c>
+      <c r="B29" s="73" t="inlineStr">
+        <is>
+          <t>연구</t>
+        </is>
+      </c>
+      <c r="C29" s="74">
+        <f>COUNTIF(L:L,"D-LAB 2실")</f>
+        <v/>
+      </c>
+      <c r="D29" s="75">
+        <f>$D$21-SUM(D24:D28)</f>
+        <v/>
+      </c>
+      <c r="E29" s="75">
+        <f>$E$21-SUM(E24:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="76">
+        <f>D29+E29</f>
+        <v/>
+      </c>
       <c r="I29" s="22" t="n">
         <v>10</v>
       </c>
@@ -4154,7 +4330,7 @@
       </c>
       <c r="L29" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업지원팀</t>
         </is>
       </c>
       <c r="M29" s="22" t="inlineStr">
@@ -4169,12 +4345,28 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="46" t="n"/>
-      <c r="F30" s="12" t="n"/>
+      <c r="A30" s="68" t="inlineStr">
+        <is>
+          <t>총합</t>
+        </is>
+      </c>
+      <c r="B30" s="69" t="n"/>
+      <c r="C30" s="70">
+        <f>SUM(C24:C29)</f>
+        <v/>
+      </c>
+      <c r="D30" s="77">
+        <f>SUM(D24:D29)</f>
+        <v/>
+      </c>
+      <c r="E30" s="77">
+        <f>SUM(E24:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="78">
+        <f>SUM(F24:F29)</f>
+        <v/>
+      </c>
       <c r="I30" s="22" t="n">
         <v>11</v>
       </c>
@@ -4190,7 +4382,7 @@
       </c>
       <c r="L30" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업지원팀</t>
         </is>
       </c>
       <c r="M30" s="22" t="inlineStr">
@@ -4401,12 +4593,12 @@
       </c>
       <c r="K36" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="L36" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>사업관리팀</t>
         </is>
       </c>
       <c r="M36" s="22" t="inlineStr">
@@ -4437,12 +4629,12 @@
       </c>
       <c r="K37" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="L37" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>사업관리팀</t>
         </is>
       </c>
       <c r="M37" s="22" t="inlineStr">
@@ -4473,12 +4665,12 @@
       </c>
       <c r="K38" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="L38" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>영업기획팀</t>
         </is>
       </c>
       <c r="M38" s="22" t="inlineStr">
@@ -4509,12 +4701,12 @@
       </c>
       <c r="K39" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="L39" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>영업기획팀</t>
         </is>
       </c>
       <c r="M39" s="22" t="inlineStr">
@@ -4545,12 +4737,12 @@
       </c>
       <c r="K40" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="L40" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>영업기획팀</t>
         </is>
       </c>
       <c r="M40" s="22" t="inlineStr">
@@ -4581,12 +4773,12 @@
       </c>
       <c r="K41" s="22" t="inlineStr">
         <is>
-          <t>사업관리본부</t>
+          <t>사업관리2실</t>
         </is>
       </c>
       <c r="L41" s="22" t="inlineStr">
         <is>
-          <t>사업관리2실</t>
+          <t>영업기획팀</t>
         </is>
       </c>
       <c r="M41" s="22" t="inlineStr">
@@ -4850,7 +5042,7 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>

</xml_diff>